<commit_message>
parsing and showing distinct ACES types
</commit_message>
<xml_diff>
--- a/adapters/outgoing/parse-file/xslx-parse-file/src/test/resources/Master Data Record for 09.05.26 Revised.xlsx
+++ b/adapters/outgoing/parse-file/xslx-parse-file/src/test/resources/Master Data Record for 09.05.26 Revised.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <fileSharing readOnlyRecommended="1"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0ECF02D-A758-BE47-8AF8-61196CDC8D42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E93F4B98-92AD-FB48-BF53-571BABB717B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34941,14 +34941,22 @@
       <c r="R3" s="147">
         <v>4</v>
       </c>
-      <c r="S3" s="147"/>
+      <c r="S3" s="147">
+        <v>2</v>
+      </c>
       <c r="T3" s="147"/>
-      <c r="U3" s="147"/>
+      <c r="U3" s="147">
+        <v>8</v>
+      </c>
       <c r="V3" s="147"/>
-      <c r="W3" s="147"/>
+      <c r="W3" s="147">
+        <v>4</v>
+      </c>
       <c r="X3" s="147"/>
       <c r="Y3" s="147"/>
-      <c r="Z3" s="147"/>
+      <c r="Z3" s="147">
+        <v>10</v>
+      </c>
       <c r="AA3" s="52"/>
       <c r="AB3" s="52"/>
       <c r="AC3" s="52"/>

</xml_diff>